<commit_message>
Add TC_11 test case configuration to Excel
Added TC_11 test case definition to OB_Automation.xlsx:
- Test Scenario: To Raise an Invoice as Vendor_Business and Pay Invoice as Client_Individual
- Credentials TC_03, TC_04: Vendor_Business
- Credentials TC_05, TC_06, TC_07, TC_08: Client_Individual
- Invoice: Vendor_Business + Client_Individual

This completes the four credential/invoice combination coverage:
- TC_01-08: Vendor_Individual + Client_Business
- TC_09: Vendor_Individual + Client_Individual
- TC_10: Vendor_Business + Client_Business
- TC_11: Vendor_Business + Client_Individual

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Testcase/OB_Automation.xlsx
+++ b/Testcase/OB_Automation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vishesh\OmneyBusiness\Testcase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26CFCF3C-A878-49E2-BCE7-733BA73A706F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355B714C-2B60-48CF-B6C4-E0153743EAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="134">
   <si>
     <t>TC_ID</t>
   </si>
@@ -479,6 +479,20 @@
   </si>
   <si>
     <t>Vendor_Business + Client_Business</t>
+  </si>
+  <si>
+    <t>Vendor_Business + Client_Individual</t>
+  </si>
+  <si>
+    <t>{Current Date +4}</t>
+  </si>
+  <si>
+    <t>To Raise and Invoice as Vendor_Business and Pay Invoice as Client_Individual</t>
+  </si>
+  <si>
+    <t>Credentials TC_03, TC_04: Vendor_Business
+Credentials TC_05, TC_06, TC_07, TC_08: Client_Individual
+Invoice: Vendor_Business + Client_Individual</t>
   </si>
 </sst>
 </file>
@@ -1090,16 +1104,32 @@
       <c r="D11" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E11" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -1425,7 +1455,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{345A23DB-58DC-46BE-9F5C-7A8F4F6C461E}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -1578,6 +1608,38 @@
         <v>68</v>
       </c>
     </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" t="s">
+        <v>106</v>
+      </c>
+      <c r="G5" t="s">
+        <v>126</v>
+      </c>
+      <c r="H5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" t="s">
+        <v>104</v>
+      </c>
+      <c r="K5" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Description and Supporting Documents fields to TC_03
- Add random description generator (max 45 chars) with numbers and special chars
- Add Description textarea filling with proper blur() for focus management
- Add Supporting Documents file upload support
- Fix Amount field focus issue by adding explicit click() before fill()
- Increase success popup detection timeout for file uploads

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Testcase/OB_Automation.xlsx
+++ b/Testcase/OB_Automation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vishesh\OmneyBusiness\Testcase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355B714C-2B60-48CF-B6C4-E0153743EAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFE7581-011F-412E-8C46-19BE0D626638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Testcase" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="142">
   <si>
     <t>TC_ID</t>
   </si>
@@ -129,9 +129,6 @@
     <t xml:space="preserve">User Pays invoice without Completing profile- P &amp; B </t>
   </si>
   <si>
-    <t>To Pay Invoice as Business</t>
-  </si>
-  <si>
     <t>To Add a Client as Business</t>
   </si>
   <si>
@@ -151,9 +148,6 @@
   </si>
   <si>
     <t>To Reject a invoice</t>
-  </si>
-  <si>
-    <t>Pay Invoice&gt;&gt; Raise New Invoice</t>
   </si>
   <si>
     <t>TC_15</t>
@@ -272,9 +266,6 @@
   </si>
   <si>
     <t>To Add a Client as Individual</t>
-  </si>
-  <si>
-    <t>To Pay Invoice as Individual</t>
   </si>
   <si>
     <t>1. Navigate to URL</t>
@@ -493,6 +484,39 @@
     <t>Credentials TC_03, TC_04: Vendor_Business
 Credentials TC_05, TC_06, TC_07, TC_08: Client_Individual
 Invoice: Vendor_Business + Client_Individual</t>
+  </si>
+  <si>
+    <t>TC_29</t>
+  </si>
+  <si>
+    <t>TC_30</t>
+  </si>
+  <si>
+    <t>TC_31</t>
+  </si>
+  <si>
+    <t>TC_32</t>
+  </si>
+  <si>
+    <t>TC_33</t>
+  </si>
+  <si>
+    <t>TC_34</t>
+  </si>
+  <si>
+    <t>TC_35</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Supporting Documents</t>
+  </si>
+  <si>
+    <t>{Random Desciption with Numbers and Special characters}</t>
+  </si>
+  <si>
+    <t>D:\Vishesh\FAB\Holiday List 2022.pdf</t>
   </si>
 </sst>
 </file>
@@ -885,7 +909,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -924,13 +948,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>8</v>
@@ -947,7 +971,7 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
@@ -961,16 +985,16 @@
         <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>8</v>
@@ -981,14 +1005,14 @@
         <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>8</v>
@@ -999,16 +1023,16 @@
         <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>8</v>
@@ -1019,13 +1043,13 @@
         <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>8</v>
@@ -1036,16 +1060,16 @@
         <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>8</v>
@@ -1056,16 +1080,16 @@
         <v>18</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>8</v>
@@ -1076,16 +1100,16 @@
         <v>19</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>8</v>
@@ -1096,16 +1120,16 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>8</v>
@@ -1116,16 +1140,16 @@
         <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>8</v>
@@ -1135,13 +1159,19 @@
       <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1152,179 +1182,175 @@
       <c r="A15" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="B15" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>76</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B24" t="s">
-        <v>32</v>
+        <v>45</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>50</v>
+      <c r="B27" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>131</v>
+      </c>
       <c r="B30" s="2" t="s">
-        <v>33</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>132</v>
+      </c>
       <c r="B31" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="B32" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>134</v>
+      </c>
       <c r="B33" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="B34" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="B35" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B39" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="40" spans="2:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="B40" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="B41" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1348,93 +1374,93 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H2" t="s">
         <v>88</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G2" t="s">
-        <v>86</v>
-      </c>
-      <c r="H2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1455,7 +1481,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{345A23DB-58DC-46BE-9F5C-7A8F4F6C461E}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -1466,178 +1492,212 @@
     <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="54.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" t="s">
         <v>54</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" t="s">
-        <v>60</v>
-      </c>
       <c r="G1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" t="s">
         <v>61</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" t="s">
         <v>63</v>
       </c>
-      <c r="I1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>65</v>
       </c>
-      <c r="K1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
         <v>55</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" t="s">
-        <v>59</v>
-      </c>
       <c r="F2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K2" t="s">
         <v>66</v>
       </c>
-      <c r="K2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L2" t="s">
+        <v>140</v>
+      </c>
+      <c r="M2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" t="s">
         <v>55</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>57</v>
       </c>
-      <c r="E3" t="s">
-        <v>59</v>
-      </c>
       <c r="F3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K3" t="s">
         <v>66</v>
       </c>
-      <c r="K3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L3" t="s">
+        <v>140</v>
+      </c>
+      <c r="M3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
         <v>55</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>57</v>
       </c>
-      <c r="E4" t="s">
-        <v>59</v>
-      </c>
       <c r="F4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G4" t="s">
+        <v>123</v>
+      </c>
+      <c r="H4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" t="s">
+        <v>101</v>
+      </c>
+      <c r="K4" t="s">
+        <v>66</v>
+      </c>
+      <c r="L4" t="s">
+        <v>140</v>
+      </c>
+      <c r="M4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F5" t="s">
         <v>103</v>
       </c>
-      <c r="G4" t="s">
-        <v>126</v>
-      </c>
-      <c r="H4" t="s">
-        <v>83</v>
-      </c>
-      <c r="I4" t="s">
-        <v>55</v>
-      </c>
-      <c r="J4" t="s">
-        <v>104</v>
-      </c>
-      <c r="K4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" t="s">
-        <v>106</v>
-      </c>
       <c r="G5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="H5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="K5" t="s">
-        <v>68</v>
+        <v>66</v>
+      </c>
+      <c r="L5" t="s">
+        <v>140</v>
+      </c>
+      <c r="M5" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>